<commit_message>
added data displaying in table - todo the push to db
</commit_message>
<xml_diff>
--- a/wordhole_records.xlsx
+++ b/wordhole_records.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leeds365-my.sharepoint.com/personal/cenpas_leeds_ac_uk/Documents/Documents/Wordle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{20ED891C-4D8D-49E3-806B-767689131E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E14882B-119E-4C90-B96D-0DC6DE4D24CD}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{20ED891C-4D8D-49E3-806B-767689131E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A151450-2866-4A82-8532-51886FCA9F1E}"/>
   <bookViews>
-    <workbookView xWindow="28755" yWindow="1545" windowWidth="27105" windowHeight="13200" xr2:uid="{0E73B5D4-4342-4984-9DBD-C032C52B68A7}"/>
+    <workbookView xWindow="690" yWindow="1500" windowWidth="23445" windowHeight="11910" xr2:uid="{0E73B5D4-4342-4984-9DBD-C032C52B68A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Round 14" sheetId="21" r:id="rId1"/>
@@ -1505,32 +1505,38 @@
         <f>IF(AD4&lt;&gt;"",AC4+AE4,"")</f>
         <v>3</v>
       </c>
-      <c r="AG4" s="38"/>
-      <c r="AH4" s="18" t="str">
+      <c r="AG4" s="38">
+        <v>4</v>
+      </c>
+      <c r="AH4" s="18">
         <f>IF(AG4&lt;&gt;"",AG4-$B$1,"")</f>
-        <v/>
-      </c>
-      <c r="AI4" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="13">
         <f>IF(AG4&lt;&gt;"",AF4+AH4,"")</f>
-        <v/>
-      </c>
-      <c r="AJ4" s="38"/>
-      <c r="AK4" s="18" t="str">
+        <v>3</v>
+      </c>
+      <c r="AJ4" s="38">
+        <v>6</v>
+      </c>
+      <c r="AK4" s="18">
         <f>IF(AJ4&lt;&gt;"",AJ4-$B$1,"")</f>
-        <v/>
-      </c>
-      <c r="AL4" s="13" t="str">
+        <v>2</v>
+      </c>
+      <c r="AL4" s="13">
         <f>IF(AJ4&lt;&gt;"",AI4+AK4,"")</f>
-        <v/>
-      </c>
-      <c r="AM4" s="38"/>
-      <c r="AN4" s="18" t="str">
+        <v>5</v>
+      </c>
+      <c r="AM4" s="38">
+        <v>4</v>
+      </c>
+      <c r="AN4" s="18">
         <f>IF(AM4&lt;&gt;"",AM4-$B$1,"")</f>
-        <v/>
-      </c>
-      <c r="AO4" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="AO4" s="13">
         <f>IF(AM4&lt;&gt;"",AL4+AN4,"")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="AP4" s="38"/>
       <c r="AQ4" s="18" t="str">
@@ -1720,23 +1726,27 @@
         <f t="shared" ref="AI5:AI9" si="21">IF(AG5&lt;&gt;"",AF5+AH5,"")</f>
         <v>2</v>
       </c>
-      <c r="AJ5" s="16"/>
-      <c r="AK5" s="2" t="str">
+      <c r="AJ5" s="16">
+        <v>4</v>
+      </c>
+      <c r="AK5" s="2">
         <f t="shared" ref="AK5:AK9" si="22">IF(AJ5&lt;&gt;"",AJ5-$B$1,"")</f>
-        <v/>
-      </c>
-      <c r="AL5" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="13">
         <f t="shared" ref="AL5:AL9" si="23">IF(AJ5&lt;&gt;"",AI5+AK5,"")</f>
-        <v/>
-      </c>
-      <c r="AM5" s="16"/>
-      <c r="AN5" s="2" t="str">
+        <v>2</v>
+      </c>
+      <c r="AM5" s="16">
+        <v>5</v>
+      </c>
+      <c r="AN5" s="2">
         <f t="shared" ref="AN5:AN9" si="24">IF(AM5&lt;&gt;"",AM5-$B$1,"")</f>
-        <v/>
-      </c>
-      <c r="AO5" s="13" t="str">
+        <v>1</v>
+      </c>
+      <c r="AO5" s="13">
         <f t="shared" ref="AO5:AO9" si="25">IF(AM5&lt;&gt;"",AL5+AN5,"")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="AP5" s="16"/>
       <c r="AQ5" s="2" t="str">
@@ -1926,23 +1936,27 @@
         <f t="shared" si="21"/>
         <v>5.0000999999999998</v>
       </c>
-      <c r="AJ6" s="16"/>
-      <c r="AK6" s="2" t="str">
+      <c r="AJ6" s="16">
+        <v>6</v>
+      </c>
+      <c r="AK6" s="2">
         <f t="shared" si="22"/>
-        <v/>
-      </c>
-      <c r="AL6" s="13" t="str">
+        <v>2</v>
+      </c>
+      <c r="AL6" s="13">
         <f t="shared" si="23"/>
-        <v/>
-      </c>
-      <c r="AM6" s="16"/>
-      <c r="AN6" s="2" t="str">
+        <v>7.0000999999999998</v>
+      </c>
+      <c r="AM6" s="16">
+        <v>5</v>
+      </c>
+      <c r="AN6" s="2">
         <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="AO6" s="13" t="str">
+        <v>1</v>
+      </c>
+      <c r="AO6" s="13">
         <f t="shared" si="25"/>
-        <v/>
+        <v>8.0000999999999998</v>
       </c>
       <c r="AP6" s="16"/>
       <c r="AQ6" s="2" t="str">
@@ -2121,32 +2135,38 @@
         <f>IF(AD7&lt;&gt;"",AC7+AE7,"")</f>
         <v>-1</v>
       </c>
-      <c r="AG7" s="16"/>
-      <c r="AH7" s="2" t="str">
+      <c r="AG7" s="16">
+        <v>3</v>
+      </c>
+      <c r="AH7" s="2">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="AI7" s="13" t="str">
+        <v>-1</v>
+      </c>
+      <c r="AI7" s="13">
         <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="AJ7" s="16"/>
-      <c r="AK7" s="2" t="str">
+        <v>-2</v>
+      </c>
+      <c r="AJ7" s="16">
+        <v>4</v>
+      </c>
+      <c r="AK7" s="2">
         <f t="shared" si="22"/>
-        <v/>
-      </c>
-      <c r="AL7" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="13">
         <f t="shared" si="23"/>
-        <v/>
-      </c>
-      <c r="AM7" s="16"/>
-      <c r="AN7" s="2" t="str">
+        <v>-2</v>
+      </c>
+      <c r="AM7" s="16">
+        <v>5</v>
+      </c>
+      <c r="AN7" s="2">
         <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="AO7" s="13" t="str">
+        <v>1</v>
+      </c>
+      <c r="AO7" s="13">
         <f t="shared" si="25"/>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="AP7" s="16"/>
       <c r="AQ7" s="2" t="str">
@@ -2336,23 +2356,27 @@
         <f t="shared" si="21"/>
         <v>2.9999000000000002</v>
       </c>
-      <c r="AJ8" s="16"/>
-      <c r="AK8" s="2" t="str">
+      <c r="AJ8" s="16">
+        <v>5</v>
+      </c>
+      <c r="AK8" s="2">
         <f t="shared" si="22"/>
-        <v/>
-      </c>
-      <c r="AL8" s="13" t="str">
+        <v>1</v>
+      </c>
+      <c r="AL8" s="13">
         <f t="shared" si="23"/>
-        <v/>
-      </c>
-      <c r="AM8" s="16"/>
-      <c r="AN8" s="2" t="str">
+        <v>3.9999000000000002</v>
+      </c>
+      <c r="AM8" s="16">
+        <v>5</v>
+      </c>
+      <c r="AN8" s="2">
         <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="AO8" s="13" t="str">
+        <v>1</v>
+      </c>
+      <c r="AO8" s="13">
         <f t="shared" si="25"/>
-        <v/>
+        <v>4.9999000000000002</v>
       </c>
       <c r="AP8" s="16"/>
       <c r="AQ8" s="2" t="str">
@@ -2536,23 +2560,27 @@
         <f t="shared" si="21"/>
         <v>-1</v>
       </c>
-      <c r="AJ9" s="16"/>
-      <c r="AK9" s="2" t="str">
+      <c r="AJ9" s="16">
+        <v>4</v>
+      </c>
+      <c r="AK9" s="2">
         <f t="shared" si="22"/>
-        <v/>
-      </c>
-      <c r="AL9" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="AL9" s="13">
         <f t="shared" si="23"/>
-        <v/>
-      </c>
-      <c r="AM9" s="16"/>
-      <c r="AN9" s="2" t="str">
+        <v>-1</v>
+      </c>
+      <c r="AM9" s="16">
+        <v>6</v>
+      </c>
+      <c r="AN9" s="2">
         <f t="shared" si="24"/>
-        <v/>
-      </c>
-      <c r="AO9" s="13" t="str">
+        <v>2</v>
+      </c>
+      <c r="AO9" s="13">
         <f t="shared" si="25"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AP9" s="16"/>
       <c r="AQ9" s="2" t="str">
@@ -2776,19 +2804,19 @@
       <c r="AF13" s="3"/>
       <c r="AG13" s="3">
         <f>IF(COUNT(AG4:AG11)&gt;0,AVERAGE(AG4:AG11),"")</f>
-        <v>3.75</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
-      <c r="AJ13" s="3" t="str">
+      <c r="AJ13" s="3">
         <f>IF(COUNT(AJ4:AJ11)&gt;0,AVERAGE(AJ4:AJ11),"")</f>
-        <v/>
+        <v>4.833333333333333</v>
       </c>
       <c r="AK13" s="3"/>
       <c r="AL13" s="3"/>
-      <c r="AM13" s="3" t="str">
+      <c r="AM13" s="3">
         <f>IF(COUNT(AM4:AM11)&gt;0,AVERAGE(AM4:AM11),"")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="AN13" s="18"/>
       <c r="AO13" s="18"/>

</xml_diff>